<commit_message>
Multiple Product Images Support
</commit_message>
<xml_diff>
--- a/cms/Playbook_AI_Batch_Template_v2.2.xlsx
+++ b/cms/Playbook_AI_Batch_Template_v2.2.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchUpload" sheetId="1" r:id="R7c72499bc40a4bf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" r:id="R7dfc09c304b74eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R0ea65d514d6743e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sports" sheetId="4" r:id="R9e53b80b9c92405e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductVariants" sheetId="5" r:id="R755254f866984b8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataDictionary" sheetId="6" r:id="Rd8375549d7574372"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchUpload" sheetId="1" r:id="Rb1fce2b8867a405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" r:id="Rc269c1659cef48d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R4323c1238c1a4179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sports" sheetId="4" r:id="R3105b39ad8a544c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductVariants" sheetId="5" r:id="Rc542cf3ba3154341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataDictionary" sheetId="6" r:id="Rd090ef2e9d2c46c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductImages" sheetId="7" r:id="R6f4bed304e1a4c9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -426,7 +427,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -441,6 +442,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor indexed="13"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF200"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0FE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -585,7 +606,7 @@
       <x:alignment vertical="bottom"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="61">
     <x:xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="bottom"/>
     </x:xf>
@@ -742,6 +763,36 @@
       <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1241,40 +1292,40 @@
       <x:c r="AI4" s="12" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="AJ4" s="41" t="str">
+      <x:c r="AJ4" s="51" t="str">
         <x:v>Profile</x:v>
       </x:c>
-      <x:c r="AK4" s="41" t="str">
+      <x:c r="AK4" s="51" t="str">
         <x:v>SnowboardWidth</x:v>
       </x:c>
-      <x:c r="AL4" s="41" t="str">
+      <x:c r="AL4" s="51" t="str">
         <x:v>TurnRadius</x:v>
       </x:c>
-      <x:c r="AM4" s="41" t="str">
+      <x:c r="AM4" s="51" t="str">
         <x:v>BootFlex</x:v>
       </x:c>
-      <x:c r="AN4" s="41" t="str">
+      <x:c r="AN4" s="51" t="str">
         <x:v>ClosureSystem</x:v>
       </x:c>
-      <x:c r="AO4" s="41" t="str">
+      <x:c r="AO4" s="51" t="str">
         <x:v>BootFlexIndex</x:v>
       </x:c>
-      <x:c r="AP4" s="41" t="str">
+      <x:c r="AP4" s="51" t="str">
         <x:v>LastWidth</x:v>
       </x:c>
-      <x:c r="AQ4" s="41" t="str">
+      <x:c r="AQ4" s="51" t="str">
         <x:v>BindingFlex</x:v>
       </x:c>
-      <x:c r="AR4" s="41" t="str">
+      <x:c r="AR4" s="51" t="str">
         <x:v>EntryStyle</x:v>
       </x:c>
-      <x:c r="AS4" s="41" t="str">
+      <x:c r="AS4" s="51" t="str">
         <x:v>Response</x:v>
       </x:c>
-      <x:c r="AT4" s="41" t="str">
+      <x:c r="AT4" s="51" t="str">
         <x:v>DINRange</x:v>
       </x:c>
-      <x:c r="AU4" s="41" t="str">
+      <x:c r="AU4" s="51" t="str">
         <x:v>BrakeWidth</x:v>
       </x:c>
     </x:row>
@@ -1314,18 +1365,18 @@
       <x:c r="AG5" s="13"/>
       <x:c r="AH5" s="13"/>
       <x:c r="AI5" s="13"/>
-      <x:c r="AJ5" s="42"/>
-      <x:c r="AK5" s="42"/>
-      <x:c r="AL5" s="42"/>
-      <x:c r="AM5" s="42"/>
-      <x:c r="AN5" s="42"/>
-      <x:c r="AO5" s="42"/>
-      <x:c r="AP5" s="42"/>
-      <x:c r="AQ5" s="42"/>
-      <x:c r="AR5" s="42"/>
-      <x:c r="AS5" s="42"/>
-      <x:c r="AT5" s="42"/>
-      <x:c r="AU5" s="42"/>
+      <x:c r="AJ5" s="52"/>
+      <x:c r="AK5" s="52"/>
+      <x:c r="AL5" s="52"/>
+      <x:c r="AM5" s="52"/>
+      <x:c r="AN5" s="52"/>
+      <x:c r="AO5" s="52"/>
+      <x:c r="AP5" s="52"/>
+      <x:c r="AQ5" s="52"/>
+      <x:c r="AR5" s="52"/>
+      <x:c r="AS5" s="52"/>
+      <x:c r="AT5" s="52"/>
+      <x:c r="AU5" s="52"/>
     </x:row>
     <x:row r="6" ht="13.550000190734863" customHeight="1">
       <x:c r="A6" s="5"/>
@@ -1516,7 +1567,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:AU1"/>
   </x:mergeCells>
-  <x:dataValidations count="19">
+  <x:dataValidations count="28">
     <x:dataValidation type="list" sqref="G5:G504">
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
@@ -1546,6 +1597,42 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AS5:AS504">
       <x:formula1>"Playful,Balanced,Precise"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="J5:J504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="L5:P504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="T5:T504">
+      <x:formula1>2000</x:formula1>
+      <x:formula2>2100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="AL5:AL504">
+      <x:formula1>5</x:formula1>
+      <x:formula2>50</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AM5:AM504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AO5:AO504">
+      <x:formula1>40</x:formula1>
+      <x:formula2>180</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="AP5:AP504">
+      <x:formula1>85</x:formula1>
+      <x:formula2>110</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AQ5:AQ504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AU5:AU504">
+      <x:formula1>50</x:formula1>
+      <x:formula2>160</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="J5:J504">
       <x:formula1>1</x:formula1>
@@ -2353,36 +2440,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="45" t="str">
+      <x:c r="A1" s="55" t="str">
         <x:v>PRODUCT VARIANTS — Add one row per available size or length. ProductID must match a BatchUpload row.</x:v>
       </x:c>
-      <x:c r="B1" s="45"/>
-      <x:c r="C1" s="45"/>
-      <x:c r="D1" s="45"/>
-      <x:c r="E1" s="45"/>
-      <x:c r="F1" s="45"/>
-      <x:c r="G1" s="45"/>
+      <x:c r="B1" s="55"/>
+      <x:c r="C1" s="55"/>
+      <x:c r="D1" s="55"/>
+      <x:c r="E1" s="55"/>
+      <x:c r="F1" s="55"/>
+      <x:c r="G1" s="55"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="50" t="str">
+      <x:c r="A4" s="60" t="str">
         <x:v>ProductVariantID</x:v>
       </x:c>
-      <x:c r="B4" s="50" t="str">
+      <x:c r="B4" s="60" t="str">
         <x:v>ProductID</x:v>
       </x:c>
-      <x:c r="C4" s="50" t="str">
+      <x:c r="C4" s="60" t="str">
         <x:v>VariantType</x:v>
       </x:c>
-      <x:c r="D4" s="50" t="str">
+      <x:c r="D4" s="60" t="str">
         <x:v>VariantValue</x:v>
       </x:c>
-      <x:c r="E4" s="50" t="str">
+      <x:c r="E4" s="60" t="str">
         <x:v>DisplayOrder</x:v>
       </x:c>
-      <x:c r="F4" s="50" t="str">
+      <x:c r="F4" s="60" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="G4" s="50" t="str">
+      <x:c r="G4" s="60" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2399,12 +2486,16 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
   </x:mergeCells>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="C5:C504">
       <x:formula1>"Size,Length"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F5:F504">
       <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="E5:E504">
+      <x:formula1>0</x:formula1>
+      <x:formula2>10000</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="E5:E504">
       <x:formula1>0</x:formula1>
@@ -2425,11 +2516,11 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="45" t="str">
+      <x:c r="A1" s="55" t="str">
         <x:v>DATA DICTIONARY — READ ONLY REFERENCE DATA. Controlled values used by the Product Builder and CMS.</x:v>
       </x:c>
-      <x:c r="B1" s="45"/>
-      <x:c r="C1" s="45"/>
+      <x:c r="B1" s="55"/>
+      <x:c r="C1" s="55"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="40"/>
@@ -2442,13 +2533,13 @@
       <x:c r="C3" s="40"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="50" t="str">
+      <x:c r="A4" s="60" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="B4" s="50" t="str">
+      <x:c r="B4" s="60" t="str">
         <x:v>AllowedValues / Format</x:v>
       </x:c>
-      <x:c r="C4" s="50" t="str">
+      <x:c r="C4" s="60" t="str">
         <x:v>Instructions</x:v>
       </x:c>
     </x:row>
@@ -2729,34 +2820,56 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="40" t="str">
-        <x:v>Sales Dashboard text</x:v>
+        <x:v>ProductImages</x:v>
       </x:c>
       <x:c r="B30" s="40" t="str">
-        <x:v>Plain text; line breaks allowed</x:v>
+        <x:v>ProductImageID|ProductID|ImageURL|AltText|ImageRole|DisplayOrder|Active</x:v>
       </x:c>
       <x:c r="C30" s="40" t="str">
-        <x:v>CustomerProfile, SellingTips, ComparisonNotes, TalkingPoints, and CommonQuestions remain editable. Follow the Product Builder prompt for content length.</x:v>
+        <x:v>Optional normalized image rows. Use ProductImages for alternates, detail images, and lifestyle images.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="40" t="str">
-        <x:v>RecommendedProductIDs</x:v>
+        <x:v>ImageRole</x:v>
       </x:c>
       <x:c r="B31" s="40" t="str">
-        <x:v>Blank</x:v>
+        <x:v>Primary|Alternate|Detail|Lifestyle</x:v>
       </x:c>
       <x:c r="C31" s="40" t="str">
-        <x:v>Do not invent IDs. Manage normalized recommendations in Playbook Admin.</x:v>
+        <x:v>Primary is the first image shown. Additional active images appear as selectable thumbnails.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="40" t="str">
+        <x:v>Sales Dashboard text</x:v>
+      </x:c>
+      <x:c r="B32" s="40" t="str">
+        <x:v>Plain text; line breaks allowed</x:v>
+      </x:c>
+      <x:c r="C32" s="40" t="str">
+        <x:v>CustomerProfile, SellingTips, ComparisonNotes, TalkingPoints, and CommonQuestions remain editable. Follow the Product Builder prompt for content length.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="40" t="str">
+        <x:v>RecommendedProductIDs</x:v>
+      </x:c>
+      <x:c r="B33" s="40" t="str">
+        <x:v>Blank</x:v>
+      </x:c>
+      <x:c r="C33" s="40" t="str">
+        <x:v>Do not invent IDs. Manage normalized recommendations in Playbook Admin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="40" t="str">
         <x:v>ProductVariants</x:v>
       </x:c>
-      <x:c r="B32" s="40" t="str">
+      <x:c r="B34" s="40" t="str">
         <x:v>One row per size or length</x:v>
       </x:c>
-      <x:c r="C32" s="40" t="str">
+      <x:c r="C34" s="40" t="str">
         <x:v>Only use after ProductID is known. ProductVariantID must be unique.</x:v>
       </x:c>
     </x:row>
@@ -2766,4 +2879,86 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="55" t="str">
+        <x:v>PRODUCT IMAGES — Optional. Add one row per extra image. The first active image is treated as primary. ProductID must match a BatchUpload row.</x:v>
+      </x:c>
+      <x:c r="B1" s="55"/>
+      <x:c r="C1" s="55"/>
+      <x:c r="D1" s="55"/>
+      <x:c r="E1" s="55"/>
+      <x:c r="F1" s="55"/>
+      <x:c r="G1" s="55"/>
+      <x:c r="H1" s="55"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="60" t="str">
+        <x:v>ProductImageID</x:v>
+      </x:c>
+      <x:c r="B4" s="60" t="str">
+        <x:v>ProductID</x:v>
+      </x:c>
+      <x:c r="C4" s="60" t="str">
+        <x:v>ImageURL</x:v>
+      </x:c>
+      <x:c r="D4" s="60" t="str">
+        <x:v>AltText</x:v>
+      </x:c>
+      <x:c r="E4" s="60" t="str">
+        <x:v>ImageRole</x:v>
+      </x:c>
+      <x:c r="F4" s="60" t="str">
+        <x:v>DisplayOrder</x:v>
+      </x:c>
+      <x:c r="G4" s="60" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="H4" s="60" t="str">
+        <x:v>LastUpdated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str"/>
+      <x:c r="B5" t="str"/>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str"/>
+      <x:c r="E5" t="str"/>
+      <x:c r="F5" t="str"/>
+      <x:c r="G5" t="str"/>
+      <x:c r="H5" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="E5:E504">
+      <x:formula1>"Primary,Alternate,Detail,Lifestyle"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G5:G504">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="F5:F504">
+      <x:formula1>0</x:formula1>
+      <x:formula2>10000</x:formula2>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Product Variants in Admin
</commit_message>
<xml_diff>
--- a/cms/Playbook_AI_Batch_Template_v2.2.xlsx
+++ b/cms/Playbook_AI_Batch_Template_v2.2.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchUpload" sheetId="1" r:id="Rb1fce2b8867a405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" r:id="Rc269c1659cef48d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R4323c1238c1a4179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sports" sheetId="4" r:id="R3105b39ad8a544c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductVariants" sheetId="5" r:id="Rc542cf3ba3154341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataDictionary" sheetId="6" r:id="Rd090ef2e9d2c46c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductImages" sheetId="7" r:id="R6f4bed304e1a4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchUpload" sheetId="1" r:id="R46b901216f0a4c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" r:id="R43bd16ca5d034167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="3" r:id="R2f74fa9fd53d4485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sports" sheetId="4" r:id="R00c5849f0ad54fd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductVariants" sheetId="5" r:id="R834db9235ca64b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataDictionary" sheetId="6" r:id="R31b95d5bff094627"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductImages" sheetId="7" r:id="R90d86c37e0184b4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -427,7 +427,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -442,6 +442,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor indexed="13"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF200"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0FE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -606,7 +626,7 @@
       <x:alignment vertical="bottom"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="61">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="bottom"/>
     </x:xf>
@@ -793,6 +813,36 @@
       <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1292,40 +1342,40 @@
       <x:c r="AI4" s="12" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="AJ4" s="51" t="str">
+      <x:c r="AJ4" s="61" t="str">
         <x:v>Profile</x:v>
       </x:c>
-      <x:c r="AK4" s="51" t="str">
+      <x:c r="AK4" s="61" t="str">
         <x:v>SnowboardWidth</x:v>
       </x:c>
-      <x:c r="AL4" s="51" t="str">
+      <x:c r="AL4" s="61" t="str">
         <x:v>TurnRadius</x:v>
       </x:c>
-      <x:c r="AM4" s="51" t="str">
+      <x:c r="AM4" s="61" t="str">
         <x:v>BootFlex</x:v>
       </x:c>
-      <x:c r="AN4" s="51" t="str">
+      <x:c r="AN4" s="61" t="str">
         <x:v>ClosureSystem</x:v>
       </x:c>
-      <x:c r="AO4" s="51" t="str">
+      <x:c r="AO4" s="61" t="str">
         <x:v>BootFlexIndex</x:v>
       </x:c>
-      <x:c r="AP4" s="51" t="str">
+      <x:c r="AP4" s="61" t="str">
         <x:v>LastWidth</x:v>
       </x:c>
-      <x:c r="AQ4" s="51" t="str">
+      <x:c r="AQ4" s="61" t="str">
         <x:v>BindingFlex</x:v>
       </x:c>
-      <x:c r="AR4" s="51" t="str">
+      <x:c r="AR4" s="61" t="str">
         <x:v>EntryStyle</x:v>
       </x:c>
-      <x:c r="AS4" s="51" t="str">
+      <x:c r="AS4" s="61" t="str">
         <x:v>Response</x:v>
       </x:c>
-      <x:c r="AT4" s="51" t="str">
+      <x:c r="AT4" s="61" t="str">
         <x:v>DINRange</x:v>
       </x:c>
-      <x:c r="AU4" s="51" t="str">
+      <x:c r="AU4" s="61" t="str">
         <x:v>BrakeWidth</x:v>
       </x:c>
     </x:row>
@@ -1365,18 +1415,18 @@
       <x:c r="AG5" s="13"/>
       <x:c r="AH5" s="13"/>
       <x:c r="AI5" s="13"/>
-      <x:c r="AJ5" s="52"/>
-      <x:c r="AK5" s="52"/>
-      <x:c r="AL5" s="52"/>
-      <x:c r="AM5" s="52"/>
-      <x:c r="AN5" s="52"/>
-      <x:c r="AO5" s="52"/>
-      <x:c r="AP5" s="52"/>
-      <x:c r="AQ5" s="52"/>
-      <x:c r="AR5" s="52"/>
-      <x:c r="AS5" s="52"/>
-      <x:c r="AT5" s="52"/>
-      <x:c r="AU5" s="52"/>
+      <x:c r="AJ5" s="62"/>
+      <x:c r="AK5" s="62"/>
+      <x:c r="AL5" s="62"/>
+      <x:c r="AM5" s="62"/>
+      <x:c r="AN5" s="62"/>
+      <x:c r="AO5" s="62"/>
+      <x:c r="AP5" s="62"/>
+      <x:c r="AQ5" s="62"/>
+      <x:c r="AR5" s="62"/>
+      <x:c r="AS5" s="62"/>
+      <x:c r="AT5" s="62"/>
+      <x:c r="AU5" s="62"/>
     </x:row>
     <x:row r="6" ht="13.550000190734863" customHeight="1">
       <x:c r="A6" s="5"/>
@@ -1567,7 +1617,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:AU1"/>
   </x:mergeCells>
-  <x:dataValidations count="28">
+  <x:dataValidations count="37">
     <x:dataValidation type="list" sqref="G5:G504">
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
@@ -1597,6 +1647,42 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AS5:AS504">
       <x:formula1>"Playful,Balanced,Precise"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="J5:J504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="L5:P504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="T5:T504">
+      <x:formula1>2000</x:formula1>
+      <x:formula2>2100</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="AL5:AL504">
+      <x:formula1>5</x:formula1>
+      <x:formula2>50</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AM5:AM504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AO5:AO504">
+      <x:formula1>40</x:formula1>
+      <x:formula2>180</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="AP5:AP504">
+      <x:formula1>85</x:formula1>
+      <x:formula2>110</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AQ5:AQ504">
+      <x:formula1>1</x:formula1>
+      <x:formula2>5</x:formula2>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="AU5:AU504">
+      <x:formula1>50</x:formula1>
+      <x:formula2>160</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="J5:J504">
       <x:formula1>1</x:formula1>
@@ -2440,36 +2526,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="55" t="str">
+      <x:c r="A1" s="65" t="str">
         <x:v>PRODUCT VARIANTS — Add one row per available size or length. ProductID must match a BatchUpload row.</x:v>
       </x:c>
-      <x:c r="B1" s="55"/>
-      <x:c r="C1" s="55"/>
-      <x:c r="D1" s="55"/>
-      <x:c r="E1" s="55"/>
-      <x:c r="F1" s="55"/>
-      <x:c r="G1" s="55"/>
+      <x:c r="B1" s="65"/>
+      <x:c r="C1" s="65"/>
+      <x:c r="D1" s="65"/>
+      <x:c r="E1" s="65"/>
+      <x:c r="F1" s="65"/>
+      <x:c r="G1" s="65"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="60" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>ProductVariantID</x:v>
       </x:c>
-      <x:c r="B4" s="60" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>ProductID</x:v>
       </x:c>
-      <x:c r="C4" s="60" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>VariantType</x:v>
       </x:c>
-      <x:c r="D4" s="60" t="str">
+      <x:c r="D4" s="70" t="str">
         <x:v>VariantValue</x:v>
       </x:c>
-      <x:c r="E4" s="60" t="str">
+      <x:c r="E4" s="70" t="str">
         <x:v>DisplayOrder</x:v>
       </x:c>
-      <x:c r="F4" s="60" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="G4" s="60" t="str">
+      <x:c r="G4" s="70" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2486,12 +2572,16 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
   </x:mergeCells>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="C5:C504">
       <x:formula1>"Size,Length"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F5:F504">
       <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="E5:E504">
+      <x:formula1>0</x:formula1>
+      <x:formula2>10000</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="E5:E504">
       <x:formula1>0</x:formula1>
@@ -2516,11 +2606,11 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="55" t="str">
+      <x:c r="A1" s="65" t="str">
         <x:v>DATA DICTIONARY — READ ONLY REFERENCE DATA. Controlled values used by the Product Builder and CMS.</x:v>
       </x:c>
-      <x:c r="B1" s="55"/>
-      <x:c r="C1" s="55"/>
+      <x:c r="B1" s="65"/>
+      <x:c r="C1" s="65"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="40"/>
@@ -2533,13 +2623,13 @@
       <x:c r="C3" s="40"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="60" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="B4" s="60" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>AllowedValues / Format</x:v>
       </x:c>
-      <x:c r="C4" s="60" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>Instructions</x:v>
       </x:c>
     </x:row>
@@ -2867,10 +2957,10 @@
         <x:v>ProductVariants</x:v>
       </x:c>
       <x:c r="B34" s="40" t="str">
-        <x:v>One row per size or length</x:v>
+        <x:v>One row per size, length, or brake width</x:v>
       </x:c>
       <x:c r="C34" s="40" t="str">
-        <x:v>Only use after ProductID is known. ProductVariantID must be unique.</x:v>
+        <x:v>Only use after ProductID is known. ProductVariantID must be unique. For ski bindings, use VariantType Brake Width and numeric VariantValue such as 95.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2896,40 +2986,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="55" t="str">
+      <x:c r="A1" s="65" t="str">
         <x:v>PRODUCT IMAGES — Optional. Add one row per extra image. The first active image is treated as primary. ProductID must match a BatchUpload row.</x:v>
       </x:c>
-      <x:c r="B1" s="55"/>
-      <x:c r="C1" s="55"/>
-      <x:c r="D1" s="55"/>
-      <x:c r="E1" s="55"/>
-      <x:c r="F1" s="55"/>
-      <x:c r="G1" s="55"/>
-      <x:c r="H1" s="55"/>
+      <x:c r="B1" s="65"/>
+      <x:c r="C1" s="65"/>
+      <x:c r="D1" s="65"/>
+      <x:c r="E1" s="65"/>
+      <x:c r="F1" s="65"/>
+      <x:c r="G1" s="65"/>
+      <x:c r="H1" s="65"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="60" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>ProductImageID</x:v>
       </x:c>
-      <x:c r="B4" s="60" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>ProductID</x:v>
       </x:c>
-      <x:c r="C4" s="60" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>ImageURL</x:v>
       </x:c>
-      <x:c r="D4" s="60" t="str">
+      <x:c r="D4" s="70" t="str">
         <x:v>AltText</x:v>
       </x:c>
-      <x:c r="E4" s="60" t="str">
+      <x:c r="E4" s="70" t="str">
         <x:v>ImageRole</x:v>
       </x:c>
-      <x:c r="F4" s="60" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>DisplayOrder</x:v>
       </x:c>
-      <x:c r="G4" s="60" t="str">
+      <x:c r="G4" s="70" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="H4" s="60" t="str">
+      <x:c r="H4" s="70" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2947,12 +3037,16 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="E5:E504">
       <x:formula1>"Primary,Alternate,Detail,Lifestyle"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G5:G504">
       <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="between" sqref="F5:F504">
+      <x:formula1>0</x:formula1>
+      <x:formula2>10000</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="F5:F504">
       <x:formula1>0</x:formula1>

</xml_diff>